<commit_message>
docs: daesun·samdong task_list에 작성가이드 시트 추가
kyungnam 예시를 참고해 분석번호별로 필요한 파라미터 시트명/컬럼/작성방법을 표로 정리.
특히 27번(감가상각_평가손익분석)은 유형자산명이 아닌 손익계정명을 적는 것이라는 점과,
감가상각_유형자산롤포워드·유형자산_처분손익 두 시트는 분석목록에 번호가 없이 27번 실행 시
Phase2/3로 자동 실행되며 비워두면 조용히 건너뛴다는 점을 명시.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015vdUxpMCVVVCt1HCN5kaBL
</commit_message>
<xml_diff>
--- a/journal_analyzer/daesun/task_list_daesun.xlsx
+++ b/journal_analyzer/daesun/task_list_daesun.xlsx
@@ -8,25 +8,26 @@
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="분석목록" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="심층분석 (계정별 Top) " sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="총계정원장" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="거래처 전기_당기 비교" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="상대계정 분석" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="벤포드 분석" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="라운드넘버 분석" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="매출 vs 비용 교차" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="잔액증감분석 (게정별 거래처벌)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="계정별 상세거래내역" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="특수관계자 분석" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="리스완전성" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="은행조회서 완전성" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="거래처분析" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="손익월별분析" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="AI계정별분석_실행" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="감가상각_평가손익분석" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="감가상각_유형자산롤포워드" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="유형자산_처분손익" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="작성가이드" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="분석목록" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="심층분석 (계정별 Top) " sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="총계정원장" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="거래처 전기_당기 비교" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="상대계정 분석" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="벤포드 분석" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="라운드넘버 분석" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="매출 vs 비용 교차" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="잔액증감분석 (게정별 거래처벌)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="계정별 상세거래내역" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="특수관계자 분석" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="리스완전성" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="은행조회서 완전성" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="거래처분析" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="손익월별분析" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="AI계정별분석_실행" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="감가상각_평가손익분석" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="감가상각_유형자산롤포워드" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="유형자산_처분손익" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,13 +39,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -67,9 +71,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,12 +524,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>계정명</t>
+          <t>구분</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>구분</t>
+          <t>계정과목</t>
         </is>
       </c>
     </row>
@@ -539,23 +544,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>계정과목</t>
+          <t>계정명</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>금액유형</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
+          <t>구분</t>
         </is>
       </c>
     </row>
@@ -570,16 +570,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>거래처명</t>
+          <t>계정과목</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
+        <is>
+          <t>금액유형</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>실행여부</t>
         </is>
@@ -602,7 +607,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>계정과목</t>
+          <t>거래처명</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -622,13 +627,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>계정과목</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
         </is>
       </c>
     </row>
@@ -643,40 +653,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>작업명</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
           <t>계정과목</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>거래처명</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>금액열</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>※ 사용법: 작업명(자유기재) / 계정과목·거래처명은 콤마로 여러 개 가능 / 금액열: 차변·대변·both / 실행여부 Y인 행만 처리됨</t>
         </is>
       </c>
     </row>
@@ -691,23 +674,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>작업명</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>계정과목</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>거래처명</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>금액열</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>실행여부</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>※ 사용법: 작업명(자유기재) / 계정과목·거래처명은 콤마로 여러 개 가능 / 금액열: 차변·대변·both / 실행여부 Y인 행만 처리됨</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -732,6 +732,11 @@
         </is>
       </c>
       <c r="B1" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>실행여부</t>
         </is>
@@ -748,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -759,22 +764,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>금액열</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>그룹기준열</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>실행여부</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>비고</t>
         </is>
       </c>
     </row>
@@ -789,41 +779,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>유형자산계정명</t>
+          <t>계정과목</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>감가상각누계액계정명</t>
+          <t>금액열</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>대체상대계정</t>
+          <t>그룹기준열</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>취득원가_수동조정</t>
+          <t>실행여부</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
-        <is>
-          <t>상각누계액_수동조정</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -840,688 +820,697 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>분석번호</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>분석명</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>설명</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>분석대상</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>기준월</t>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>파라미터 시트명</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>필요 컬럼</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>작성방법</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>비고</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>거래처 전기_당기 비교</t>
+          <t>(공통)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>전기/당기 거래처별 금액 비교 → 거래처비교 시트 참조</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>분석목록 시트의 '분석명'은 아래 파라미터 시트명과 철자가 정확히 같아야 연결됩니다 (예: 분석명 '벤포드 분석' ↔ 시트명 '벤포드 분석'). 파라미터 시트 내 '실행여부' 열이 있는 경우 그 열이 Y(또는 O)인 행만 처리되고, 없는 시트는 적힌 행 전부가 처리됩니다.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>분석목록 자체의 실행여부는 메뉴 On/Off, 파라미터 시트의 실행여부는 그 메뉴 내 항목별 On/Off</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>벤포드 분석</t>
+          <t>거래처 전기_당기 비교</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>첫째자리 빈도 벤포드 기댓값 비교 → 벤포드분석 시트 참조</t>
+          <t>계정과목 / 금액열(차변·대변·both) / 실행여부 / 비고</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>계정과목 한 줄에 하나씩. 지정한 방향(차변/대변)의 거래처별 전기·당기 금액을 비교표로 생성</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>데이터 개요</t>
+          <t>벤포드 분석</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>전체 데이터 건수/금액 요약 (파라미터 불필요)</t>
+          <t>계정과목 / 금액열 / 실행여부 / 비고</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>벤포드 법칙을 적용할 계정·방향 지정. 데이터 5건 미만이면 자동으로 "데이터 부족" 처리</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>계정명 리스트</t>
+          <t>(파라미터 시트 없음)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>계정명 목록 및 금액 통계 (파라미터 불필요)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>분석목록에서 실행여부만 Y로 두면 전체 데이터 요약이 자동 생성됨</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>파라미터 불필요</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>사원별 집계</t>
+          <t>(파라미터 시트 없음)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>사원별 차변/대변 계정 집계 (파라미터 불필요)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>분석목록에서 실행여부만 Y로 두면 계정명 목록·통계가 자동 생성됨</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>파라미터 불필요</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>일자차이 분석</t>
+          <t>(파라미터 시트 없음)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>전표일자 vs 등록일자 N일 이상 지연 전표 → 일자차이분석 시트 참조</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>사원명 컬럼을 자동 탐지해 집계 (컬럼명이 "사원명"이 아니면 preprocess.py에서 먼저 매핑 필요)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>파라미터 불필요</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>상대계정 분석</t>
+          <t>일자차이 분석 (시트 미생성)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>특정 계정의 상대계정 분석 → 상대계정분석 시트 참조</t>
+          <t>기준일수 / 실행여부</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>쓰려면 시트명을 정확히 '일자차이 분석'으로 새로 만들고 기준일수(예: 30) 입력. 전표일자 대비 등록일자가 그 일수 이상 지연된 전표를 추출</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>등록일자 계열 컬럼이 있어야 동작</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>키워드 검색</t>
+          <t>상대계정 분석</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>적요 키워드 검색 → 키워드검색 시트 참조</t>
+          <t>계정과목 / 금액열 / 그룹기준열 / 실행여부 / 비고</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>그룹기준열은 비워두면 전표그룹키(같은 전표를 묶는 내부 키)를 자동 사용 — 보통 비워두는 게 안전</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>라운드넘버 분석</t>
+          <t>키워드검색 (시트 미생성)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>특정 배수 단위 금액 탐지 → 라운드넘버 시트 참조</t>
+          <t>키워드 / 실행여부</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>쓰려면 시트명을 정확히 '키워드검색'으로 새로 만들고 키워드를 한 줄씩 입력 (적요 컬럼에서 검색)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>특수관계자 분석</t>
+          <t>라운드넘버 분석</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>특수관계자 거래처 거래 추출 → 특수관계자 시트 참조</t>
+          <t>계정과목 / 금액열 / 최소금액 / 실행여부 / 비고</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>전체</t>
-        </is>
-      </c>
+          <t>계정과목에 '(전체)' 입력 시 전 계정 대상. 최소금액 이상 배수(10만/50만/100만/500만/1000만원)만 라운드로 탐지</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>자산 vs 부채 교차</t>
+          <t>특수관계자 분석</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>자산/부채 동시 발생 거래처 분석</t>
+          <t>거래처명 / 실행여부</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>거래처명은 부분일치 검색 (예: "판타지오" 입력 시 "(주)판타지오"도 매칭)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>매출 vs 비용 교차</t>
+          <t>자산 vs 부채 교차 (시트 미생성)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>매출/비용 동시 발생 거래처 분석</t>
+          <t>구분(자산/부채) / 계정과목</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>쓰려면 시트명을 정확히 '자산 vs 부채 교차'로 새로 만들고, 구분별 계정과목을 한 줄씩 입력</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>같은 거래처에서 자산·부채 계정이 동시에 발생하는 경우 추출</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>심층분석 (계정별 Top)</t>
+          <t>매출 vs 비용 교차</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>계정별 거래처 Top N 추출 → 심층분석 시트 참조</t>
+          <t>구분(매출/비용) / 계정과목</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>구분별로 계정과목을 한 줄씩 입력. 같은 거래처에서 매출·비용이 동시에 발생하는 경우를 찾음</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AI 계정별 분석</t>
+          <t xml:space="preserve">심층분석 (계정별 Top) </t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>계정별 월별 추이 및 샘플 추출 → AI계정별분석 시트 참조</t>
+          <t>계정과목 (선택: 개수 / 금액열 열 추가 가능)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>계정과목만 한 줄씩 나열해도 동작 (기본값: 상위 10건, 차대변 모두). 열을 추가하면 개수·방향 지정 가능</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>열 이름은 정확히 '개수', '금액열'</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>데이터·헤더 확인</t>
+          <t>AI계정별분석 (시트 미생성)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>컬럼 인식 현황 점검 (파라미터 불필요)</t>
+          <t>계정과목 / 실행여부</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>쓰려면 시트명을 정확히 'AI계정별분석'으로 새로 만들고 계정과목 입력. Gemini 호출 없이 월별추이·샘플만 추출(26번과 형식은 같으나 AI 분석은 안 함)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>거래처 분석</t>
+          <t>(파라미터 시트 없음)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>특정 거래처 복합조건 상세 분석 → 거래처분석 시트 참조</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>컬럼 인식 현황(O/X) 점검용. 실데이터 넣고 가장 먼저 돌려보면 좋음</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>파라미터 불필요</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>벤포드 이탈 상세 추출</t>
+          <t>거래처분析</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>벤포드 이탈 전표 상세 추출 → 벤포드이탈 시트 참조</t>
+          <t>작업명 / 계정과목 / 거래처명 / 금액열 / 실행여부</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>작업명은 자유 기재. 계정과목·거래처명은 콤마로 여러 개 지정 가능</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>월별 전계정 분석</t>
+          <t>벤포드이탈 (시트 미생성)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>전 계정 월별 차변/대변 집계 (파라미터 불필요)</t>
+          <t>계정과목 / 금액열 / 임계값 / 최대건수 / 실행여부</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>쓰려면 시트명을 정확히 '벤포드이탈'로 새로 만들 것. 벤포드 법칙에서 크게 벗어난 전표를 상세 추출</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>잔액증감분석 (계정별 거래처별)</t>
+          <t>(파라미터 시트 없음)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>각 계정별 거래처별로 기초잔액 증가 감소 기말 잔액 추출</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>전 계정 월별 차변/대변 집계가 자동 생성됨</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>당기</t>
+          <t>파라미터 불필요</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>총계정원장</t>
+          <t>잔액증감분석 (게정별 거래처벌)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>전기/당기/전당기 기간의 계정별 월별합계 차/대/전체로 추출</t>
+          <t>계정명 / 구분(차변·대변 또는 자산·부채)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>data/previous 폴더에 전기 "계정별_거래처별명세" 파일이 있어야 기초잔액이 채워짐 (없으면 오류 시트만 생성)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>은행조회서 완전성</t>
+          <t>총계정원장</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>이자비용, 장단기차입금, 전환사채, RCPS등의 거래처와 은행조회서 발송내역 비교</t>
+          <t>구분 / 계정과목</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>구분은 시트명 접두어로만 쓰이는 자유 기재 항목(예: 자산/부채). data에 연도가 2개 이상 섞여 있으면 연도비교 표로 자동 전환</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>계정별 상세거래내역</t>
+          <t>은행조회서 완전성</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>각 계정별로 계정과목 차변/대변/차변대변모두 를 선택하여 데이터추출</t>
+          <t>계정과목</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>비워두면 기본 계정(이자비용/단기차입금/장기차입금/전환사채 등)을 자동 사용</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>리스완전성</t>
+          <t>계정별 상세거래내역</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>K-IFRS 116호 리스 인식 대상 완전성 검토</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>계정과목 / 금액유형(차변·대변·차변대변모두) / 실행여부</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>손익월별분析</t>
+          <t>리스완전성</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>손익 계정별 전기/당기 차변·대변 선택 비교 (월별 + 거래처별)</t>
+          <t>계정과목 / 실행여부</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>비워두면 기본 계정(임차료/지급수수료/차량유지비/건물관리비/렌탈)을 자동 사용</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>전체</t>
+          <t>결과는 별도 파일로 저장됨</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AI계정별분석_실행</t>
+          <t>손익월별分析</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>계정별 월별 추이 및 샘플을 Gemini로 분석실행(15번 메뉴와 관계없이 독립 실행)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>당기</t>
-        </is>
-      </c>
+          <t>계정과목 / 구분(차변·대변·both) / 실행여부</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>AI계정별분석_실행</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>계정과목 / 실행여부</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>.env에 GEMINI_API_KEY 필요 (Gemini 실제 호출, 비용 발생)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
         <v>27</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>감가상각_평가손익분석</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>감가상각비 등 손익계정의 상대계정(자산 누계액 등) 금액을 8번과 동일 로직으로 추출 (Phase 1)</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>당기</t>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>계정과목 / 금액열 / 그룹기준열 / 실행여부 / 비고</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>★계정과목에는 유형자산명이 아니라 '손익 계정명'을 적음 (예: 감가상각비, 외화환산손익, 평가손익, 대손상각비). 8번 상대계정분석과 완전히 동일한 로직(Phase 1)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>유형자산 롤포워드/처분손익은 아래 두 시트로 별도 제어</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>27-Phase2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>감가상각_유형자산롤포워드</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>유형자산계정명 / 감가상각누계액계정명 / 대체상대계정 / 취득원가_수동조정 / 상각누계액_수동조정 / 실행여부 / 비고</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>27번이 실행여부 Y이고 이 시트에서 실행여부 Y인 행이 있으면 자동 실행됨 (분석목록에 별도 번호 없음). 대체상대계정은 계정대체가 있을 때만 입력(콤마로 여러 개 가능), 없으면 비워둠. 수동조정 2종은 전표매칭으로 못 잡는 잔여차이를 감사인이 직접 숫자로 입력(기본 0)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>비워두면(실행여부 Y행 0개) 조용히 건너뛰고 27번은 Phase1만 결과로 나옴 — 에러 아님</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>27-Phase3</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>유형자산_처분손익</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>처분이익계정명 / 처분손실계정명 / 실행여부 / 비고</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>27번 + 위 롤포워드 시트가 모두 있어야 자동 실행됨. 처분이익·처분손실 계정이 등장한 전표마다 같은 전표의 유형자산 취득원가·감가상각누계액을 찾아 처분 건별로 한 줄씩 명세 생성</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>개별 자산이 아닌 계정과목×전표 단위로만 구분됨 — 한 전표에 여러 자산을 묶어 처분하면 한 줄로 잡힘</t>
         </is>
       </c>
     </row>
@@ -1536,6 +1525,57 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>유형자산계정명</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>감가상각누계액계정명</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>대체상대계정</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>취득원가_수동조정</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>상각누계액_수동조정</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -1572,13 +1612,688 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>계정과목</t>
+          <t>분석번호</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>분석명</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>분석대상</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>기준월</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>거래처 전기_당기 비교</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>전기/당기 거래처별 금액 비교 → 거래처비교 시트 참조</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>벤포드 분석</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>첫째자리 빈도 벤포드 기댓값 비교 → 벤포드분석 시트 참조</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>데이터 개요</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>전체 데이터 건수/금액 요약 (파라미터 불필요)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>계정명 리스트</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>계정명 목록 및 금액 통계 (파라미터 불필요)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>사원별 집계</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>사원별 차변/대변 계정 집계 (파라미터 불필요)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>일자차이 분석</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>전표일자 vs 등록일자 N일 이상 지연 전표 → 일자차이분석 시트 참조</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>상대계정 분석</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>특정 계정의 상대계정 분석 → 상대계정분석 시트 참조</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>키워드 검색</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>적요 키워드 검색 → 키워드검색 시트 참조</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>라운드넘버 분석</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>특정 배수 단위 금액 탐지 → 라운드넘버 시트 참조</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>특수관계자 분석</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>특수관계자 거래처 거래 추출 → 특수관계자 시트 참조</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>자산 vs 부채 교차</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>자산/부채 동시 발생 거래처 분석</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>매출 vs 비용 교차</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>매출/비용 동시 발생 거래처 분석</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>심층분석 (계정별 Top)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>계정별 거래처 Top N 추출 → 심층분석 시트 참조</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>AI 계정별 분석</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>계정별 월별 추이 및 샘플 추출 → AI계정별분석 시트 참조</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>데이터·헤더 확인</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>컬럼 인식 현황 점검 (파라미터 불필요)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>거래처 분석</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>특정 거래처 복합조건 상세 분석 → 거래처분석 시트 참조</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>벤포드 이탈 상세 추출</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>벤포드 이탈 전표 상세 추출 → 벤포드이탈 시트 참조</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>월별 전계정 분석</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>전 계정 월별 차변/대변 집계 (파라미터 불필요)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>20</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>잔액증감분석 (계정별 거래처별)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>각 계정별 거래처별로 기초잔액 증가 감소 기말 잔액 추출</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>21</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>총계정원장</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>전기/당기/전당기 기간의 계정별 월별합계 차/대/전체로 추출</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>22</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>은행조회서 완전성</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>이자비용, 장단기차입금, 전환사채, RCPS등의 거래처와 은행조회서 발송내역 비교</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>23</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>계정별 상세거래내역</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>각 계정별로 계정과목 차변/대변/차변대변모두 를 선택하여 데이터추출</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>24</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>리스완전성</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>K-IFRS 116호 리스 인식 대상 완전성 검토</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>25</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>손익월별분析</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>손익 계정별 전기/당기 차변·대변 선택 비교 (월별 + 거래처별)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>26</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>AI계정별분석_실행</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>계정별 월별 추이 및 샘플을 Gemini로 분석실행(15번 메뉴와 관계없이 독립 실행)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>당기</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>27</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>감가상각_평가손익분석</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>감가상각비 등 손익계정의 상대계정(자산 누계액 등) 금액을 8번과 동일 로직으로 추출 (Phase 1)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>당기</t>
         </is>
       </c>
     </row>
@@ -1593,16 +2308,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
-        <is>
-          <t>구분</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
         <is>
           <t>계정과목</t>
         </is>
@@ -1619,28 +2329,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>계정과목</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>금액열</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>비고</t>
         </is>
       </c>
     </row>
@@ -1655,7 +2355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1671,15 +2371,10 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>그룹기준열</t>
+          <t>실행여부</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -1696,7 +2391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1712,10 +2407,15 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>그룹기준열</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>실행여부</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -1732,7 +2432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1748,62 +2448,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>최소금액</t>
+          <t>실행여부</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>실행여부</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t>비고</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>(전체)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>차변</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1000000000</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>10억원 이상 라운드 수 탐지</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>(전체)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>대변</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1000000000</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>N</t>
         </is>
       </c>
     </row>
@@ -1818,18 +2468,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>구분</t>
+          <t>계정과목</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>계정과목</t>
+          <t>금액열</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>최소금액</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>실행여부</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>(전체)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>10억원 이상 라운드 수 탐지</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>(전체)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>

</xml_diff>